<commit_message>
Adiciona projeto de testes de carga com Locust e WordPress
</commit_message>
<xml_diff>
--- a/resultados/resumo_resultados.xlsx
+++ b/resultados/resumo_resultados.xlsx
@@ -543,7 +543,7 @@
         <v>50</v>
       </c>
       <c r="G2" t="n">
-        <v>3789</v>
+        <v>5956</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -552,22 +552,22 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>909.5152270124188</v>
+        <v>585.601223384171</v>
       </c>
       <c r="K2" t="n">
-        <v>810</v>
+        <v>670</v>
       </c>
       <c r="L2" t="n">
-        <v>1700</v>
+        <v>1300</v>
       </c>
       <c r="M2" t="n">
-        <v>220.6885230007174</v>
+        <v>15.89835900085745</v>
       </c>
       <c r="N2" t="n">
-        <v>3123.90825500006</v>
+        <v>1969.615001999045</v>
       </c>
       <c r="O2" t="n">
-        <v>31.6999908038973</v>
+        <v>49.99484431759415</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -601,10 +601,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G3" t="n">
-        <v>3855</v>
+        <v>6715</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -613,22 +613,22 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>5313.791748194284</v>
+        <v>2213.76436484808</v>
       </c>
       <c r="K3" t="n">
-        <v>5000</v>
+        <v>2800</v>
       </c>
       <c r="L3" t="n">
-        <v>8600</v>
+        <v>4600</v>
       </c>
       <c r="M3" t="n">
-        <v>1644.180356000106</v>
+        <v>17.14072700087854</v>
       </c>
       <c r="N3" t="n">
-        <v>13645.75651899941</v>
+        <v>6949.323208000351</v>
       </c>
       <c r="O3" t="n">
-        <v>32.26939855425486</v>
+        <v>56.12025889590919</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -662,37 +662,37 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G4" t="n">
-        <v>4269</v>
+        <v>7035</v>
       </c>
       <c r="H4" t="n">
-        <v>284</v>
+        <v>234</v>
       </c>
       <c r="I4" t="n">
-        <v>6.652611852892949</v>
+        <v>3.326226012793177</v>
       </c>
       <c r="J4" t="n">
-        <v>12585.60963997846</v>
+        <v>3863.949924405379</v>
       </c>
       <c r="K4" t="n">
-        <v>14000</v>
+        <v>4500</v>
       </c>
       <c r="L4" t="n">
-        <v>16000</v>
+        <v>6900</v>
       </c>
       <c r="M4" t="n">
-        <v>2.139662999979919</v>
+        <v>1.933019999341923</v>
       </c>
       <c r="N4" t="n">
-        <v>18254.72377999995</v>
+        <v>9639.529861000485</v>
       </c>
       <c r="O4" t="n">
-        <v>35.6520984500095</v>
+        <v>58.9474631017795</v>
       </c>
       <c r="P4" t="n">
-        <v>2.371795727290396</v>
+        <v>1.960725851573049</v>
       </c>
       <c r="Q4" t="n">
         <v>2</v>
@@ -726,7 +726,7 @@
         <v>50</v>
       </c>
       <c r="G5" t="n">
-        <v>4147</v>
+        <v>6128</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -735,22 +735,22 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>761.9203371748263</v>
+        <v>566.6298279329326</v>
       </c>
       <c r="K5" t="n">
-        <v>730</v>
+        <v>660</v>
       </c>
       <c r="L5" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="M5" t="n">
-        <v>210.539489000439</v>
+        <v>15.77754899881256</v>
       </c>
       <c r="N5" t="n">
-        <v>1631.413033999706</v>
+        <v>2054.602387999694</v>
       </c>
       <c r="O5" t="n">
-        <v>34.62814539281465</v>
+        <v>51.38227345299623</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -784,10 +784,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G6" t="n">
-        <v>4612</v>
+        <v>6648</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -796,22 +796,22 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>4341.383853069809</v>
+        <v>2226.292447509765</v>
       </c>
       <c r="K6" t="n">
-        <v>4300</v>
+        <v>2800</v>
       </c>
       <c r="L6" t="n">
-        <v>6100</v>
+        <v>4600</v>
       </c>
       <c r="M6" t="n">
-        <v>517.1853000001647</v>
+        <v>14.95588900070288</v>
       </c>
       <c r="N6" t="n">
-        <v>10003.55599500017</v>
+        <v>6645.285221000449</v>
       </c>
       <c r="O6" t="n">
-        <v>38.54962147092984</v>
+        <v>55.82598333799472</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
@@ -845,37 +845,37 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G7" t="n">
-        <v>4946</v>
+        <v>7035</v>
       </c>
       <c r="H7" t="n">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="I7" t="n">
-        <v>2.911443590780429</v>
+        <v>2.388059701492538</v>
       </c>
       <c r="J7" t="n">
-        <v>10895.12334084982</v>
+        <v>3876.446723374413</v>
       </c>
       <c r="K7" t="n">
-        <v>12000</v>
+        <v>4500</v>
       </c>
       <c r="L7" t="n">
-        <v>14000</v>
+        <v>6800</v>
       </c>
       <c r="M7" t="n">
-        <v>2.173656999730156</v>
+        <v>1.997891000428353</v>
       </c>
       <c r="N7" t="n">
-        <v>15627.69980400026</v>
+        <v>9389.68379400103</v>
       </c>
       <c r="O7" t="n">
-        <v>41.4243845940105</v>
+        <v>59.00885191314532</v>
       </c>
       <c r="P7" t="n">
-        <v>1.206047590282554</v>
+        <v>1.409166612851232</v>
       </c>
       <c r="Q7" t="n">
         <v>2</v>
@@ -909,7 +909,7 @@
         <v>50</v>
       </c>
       <c r="G8" t="n">
-        <v>4026</v>
+        <v>6043</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -918,22 +918,22 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>793.3062952737301</v>
+        <v>572.8714580066244</v>
       </c>
       <c r="K8" t="n">
-        <v>750</v>
+        <v>650</v>
       </c>
       <c r="L8" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="M8" t="n">
-        <v>267.1841519995724</v>
+        <v>17.19194899851573</v>
       </c>
       <c r="N8" t="n">
-        <v>4192.741134999778</v>
+        <v>4379.5166480013</v>
       </c>
       <c r="O8" t="n">
-        <v>33.83382578340664</v>
+        <v>50.63876996951238</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
@@ -967,10 +967,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G9" t="n">
-        <v>4642</v>
+        <v>6675</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -979,22 +979,22 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>4278.667044434065</v>
+        <v>2238.193534165384</v>
       </c>
       <c r="K9" t="n">
-        <v>4300</v>
+        <v>2800</v>
       </c>
       <c r="L9" t="n">
-        <v>5900</v>
+        <v>4600</v>
       </c>
       <c r="M9" t="n">
-        <v>454.1080459994191</v>
+        <v>15.58686700082035</v>
       </c>
       <c r="N9" t="n">
-        <v>8752.087401999233</v>
+        <v>7588.980083000933</v>
       </c>
       <c r="O9" t="n">
-        <v>38.99330727043515</v>
+        <v>55.80799155046008</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -1028,37 +1028,37 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G10" t="n">
-        <v>4836</v>
+        <v>7131</v>
       </c>
       <c r="H10" t="n">
-        <v>130</v>
+        <v>239</v>
       </c>
       <c r="I10" t="n">
-        <v>2.688172043010753</v>
+        <v>3.351563595568644</v>
       </c>
       <c r="J10" t="n">
-        <v>11150.32072686806</v>
+        <v>3822.631092104337</v>
       </c>
       <c r="K10" t="n">
-        <v>12000</v>
+        <v>4500</v>
       </c>
       <c r="L10" t="n">
-        <v>14000</v>
+        <v>6800</v>
       </c>
       <c r="M10" t="n">
-        <v>2.296560999639041</v>
+        <v>2.044225999270566</v>
       </c>
       <c r="N10" t="n">
-        <v>16764.46585999929</v>
+        <v>10028.26492700115</v>
       </c>
       <c r="O10" t="n">
-        <v>40.46410224829778</v>
+        <v>59.49061956259124</v>
       </c>
       <c r="P10" t="n">
-        <v>1.087744684094027</v>
+        <v>1.993865948038046</v>
       </c>
       <c r="Q10" t="n">
         <v>2</v>
@@ -1092,7 +1092,7 @@
         <v>50</v>
       </c>
       <c r="G11" t="n">
-        <v>2590</v>
+        <v>4830</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1101,22 +1101,22 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>279.8952414359064</v>
+        <v>222.6229149766164</v>
       </c>
       <c r="K11" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="L11" t="n">
-        <v>510</v>
+        <v>580</v>
       </c>
       <c r="M11" t="n">
-        <v>121.2717839998732</v>
+        <v>14.11524299874145</v>
       </c>
       <c r="N11" t="n">
-        <v>1053.862876000039</v>
+        <v>1196.211124000911</v>
       </c>
       <c r="O11" t="n">
-        <v>21.76201319812508</v>
+        <v>40.43411573443949</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
@@ -1150,10 +1150,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G12" t="n">
-        <v>4605</v>
+        <v>7635</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -1162,22 +1162,22 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>3054.140466395015</v>
+        <v>1299.995648411648</v>
       </c>
       <c r="K12" t="n">
-        <v>2900</v>
+        <v>950</v>
       </c>
       <c r="L12" t="n">
-        <v>4800</v>
+        <v>3000</v>
       </c>
       <c r="M12" t="n">
-        <v>600.1465119998102</v>
+        <v>19.98055100011697</v>
       </c>
       <c r="N12" t="n">
-        <v>9399.49753799965</v>
+        <v>5912.170678999246</v>
       </c>
       <c r="O12" t="n">
-        <v>38.46345617477557</v>
+        <v>63.71371233157482</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -1211,10 +1211,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G13" t="n">
-        <v>4068</v>
+        <v>7664</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -1223,22 +1223,22 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>12056.11723777165</v>
+        <v>2937.128144028179</v>
       </c>
       <c r="K13" t="n">
-        <v>12000</v>
+        <v>2300</v>
       </c>
       <c r="L13" t="n">
-        <v>17000</v>
+        <v>6100</v>
       </c>
       <c r="M13" t="n">
-        <v>2647.994228000244</v>
+        <v>62.21851100053755</v>
       </c>
       <c r="N13" t="n">
-        <v>18683.69035800015</v>
+        <v>9809.897368000748</v>
       </c>
       <c r="O13" t="n">
-        <v>33.96162432867316</v>
+        <v>64.20989758131353</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -1275,7 +1275,7 @@
         <v>50</v>
       </c>
       <c r="G14" t="n">
-        <v>2586</v>
+        <v>4895</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -1284,22 +1284,22 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>284.650921709992</v>
+        <v>210.7456397838618</v>
       </c>
       <c r="K14" t="n">
-        <v>250</v>
+        <v>170</v>
       </c>
       <c r="L14" t="n">
-        <v>530</v>
+        <v>560</v>
       </c>
       <c r="M14" t="n">
-        <v>131.1812860003556</v>
+        <v>13.48364900150045</v>
       </c>
       <c r="N14" t="n">
-        <v>924.5400079998944</v>
+        <v>922.3283299998002</v>
       </c>
       <c r="O14" t="n">
-        <v>21.7203702920307</v>
+        <v>41.02703373424501</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
@@ -1333,10 +1333,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G15" t="n">
-        <v>4769</v>
+        <v>7683</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -1345,22 +1345,22 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>2840.929733678964</v>
+        <v>1289.03854716608</v>
       </c>
       <c r="K15" t="n">
-        <v>2800</v>
+        <v>960</v>
       </c>
       <c r="L15" t="n">
-        <v>4100</v>
+        <v>3100</v>
       </c>
       <c r="M15" t="n">
-        <v>388.8462120003169</v>
+        <v>17.51616799992917</v>
       </c>
       <c r="N15" t="n">
-        <v>6339.62667600008</v>
+        <v>4690.419086000475</v>
       </c>
       <c r="O15" t="n">
-        <v>40.01135880010513</v>
+        <v>64.25223764704181</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
@@ -1394,37 +1394,37 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G16" t="n">
-        <v>4828</v>
+        <v>7582</v>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I16" t="n">
-        <v>0.02071251035625518</v>
+        <v>0.09232392508572936</v>
       </c>
       <c r="J16" t="n">
-        <v>9938.821573920466</v>
+        <v>2968.885051797154</v>
       </c>
       <c r="K16" t="n">
-        <v>10000</v>
+        <v>2500</v>
       </c>
       <c r="L16" t="n">
-        <v>12000</v>
+        <v>6200</v>
       </c>
       <c r="M16" t="n">
-        <v>2.279041000292636</v>
+        <v>2.677335000043968</v>
       </c>
       <c r="N16" t="n">
-        <v>13377.27475999964</v>
+        <v>8956.47969699894</v>
       </c>
       <c r="O16" t="n">
-        <v>40.40044756772039</v>
+        <v>63.52895525453768</v>
       </c>
       <c r="P16" t="n">
-        <v>0.008367946886437499</v>
+        <v>0.0586524250569458</v>
       </c>
       <c r="Q16" t="n">
         <v>2</v>
@@ -1458,7 +1458,7 @@
         <v>50</v>
       </c>
       <c r="G17" t="n">
-        <v>2513</v>
+        <v>4815</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1467,22 +1467,22 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>357.9302145957034</v>
+        <v>232.5851011389504</v>
       </c>
       <c r="K17" t="n">
-        <v>290</v>
+        <v>180</v>
       </c>
       <c r="L17" t="n">
-        <v>690</v>
+        <v>590</v>
       </c>
       <c r="M17" t="n">
-        <v>130.1502589994925</v>
+        <v>14.36456100054784</v>
       </c>
       <c r="N17" t="n">
-        <v>3720.991485000013</v>
+        <v>4344.138362999729</v>
       </c>
       <c r="O17" t="n">
-        <v>21.14162557829327</v>
+        <v>40.34541381478859</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
@@ -1516,10 +1516,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G18" t="n">
-        <v>4312</v>
+        <v>7663</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -1528,22 +1528,22 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>3366.897302788492</v>
+        <v>1281.295474329744</v>
       </c>
       <c r="K18" t="n">
-        <v>3100</v>
+        <v>1100</v>
       </c>
       <c r="L18" t="n">
-        <v>5800</v>
+        <v>3000</v>
       </c>
       <c r="M18" t="n">
-        <v>375.5039699999543</v>
+        <v>23.26894600082596</v>
       </c>
       <c r="N18" t="n">
-        <v>8434.249889999592</v>
+        <v>6087.860371000716</v>
       </c>
       <c r="O18" t="n">
-        <v>36.18431340297757</v>
+        <v>64.37348442786221</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1577,10 +1577,10 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G19" t="n">
-        <v>5097</v>
+        <v>7740</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -1589,22 +1589,22 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>9339.818966982732</v>
+        <v>2900.48523903076</v>
       </c>
       <c r="K19" t="n">
-        <v>9700</v>
+        <v>2200</v>
       </c>
       <c r="L19" t="n">
-        <v>11000</v>
+        <v>6000</v>
       </c>
       <c r="M19" t="n">
-        <v>1652.634897000098</v>
+        <v>78.16349700078717</v>
       </c>
       <c r="N19" t="n">
-        <v>13929.43046399978</v>
+        <v>8589.768133000689</v>
       </c>
       <c r="O19" t="n">
-        <v>42.48676295266686</v>
+        <v>64.9120103683218</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -1641,7 +1641,7 @@
         <v>50</v>
       </c>
       <c r="G20" t="n">
-        <v>2606</v>
+        <v>4926</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1650,22 +1650,22 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>263.0607428791252</v>
+        <v>196.1443643442996</v>
       </c>
       <c r="K20" t="n">
-        <v>230</v>
+        <v>160</v>
       </c>
       <c r="L20" t="n">
-        <v>490</v>
+        <v>550</v>
       </c>
       <c r="M20" t="n">
-        <v>128.8428289999501</v>
+        <v>10.09824200082221</v>
       </c>
       <c r="N20" t="n">
-        <v>817.5626199999897</v>
+        <v>1106.843666999339</v>
       </c>
       <c r="O20" t="n">
-        <v>21.89612355969669</v>
+        <v>41.29322240721226</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -1699,10 +1699,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G21" t="n">
-        <v>4886</v>
+        <v>8097</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1711,22 +1711,22 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>2768.890315367793</v>
+        <v>1169.689412981093</v>
       </c>
       <c r="K21" t="n">
-        <v>2600</v>
+        <v>980</v>
       </c>
       <c r="L21" t="n">
-        <v>4300</v>
+        <v>2800</v>
       </c>
       <c r="M21" t="n">
-        <v>542.3206960003881</v>
+        <v>12.29028099987772</v>
       </c>
       <c r="N21" t="n">
-        <v>6784.778703000484</v>
+        <v>4684.626930000377</v>
       </c>
       <c r="O21" t="n">
-        <v>40.85630664500072</v>
+        <v>67.59115360186853</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
@@ -1760,10 +1760,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G22" t="n">
-        <v>5217</v>
+        <v>8437</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1772,22 +1772,22 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>9035.658456239236</v>
+        <v>2590.249674089247</v>
       </c>
       <c r="K22" t="n">
-        <v>9400</v>
+        <v>2200</v>
       </c>
       <c r="L22" t="n">
-        <v>10000</v>
+        <v>5500</v>
       </c>
       <c r="M22" t="n">
-        <v>2187.802553999973</v>
+        <v>14.8147580002842</v>
       </c>
       <c r="N22" t="n">
-        <v>12397.30124500056</v>
+        <v>7995.809256000939</v>
       </c>
       <c r="O22" t="n">
-        <v>43.56675960186814</v>
+        <v>70.40594511932927</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
@@ -1824,7 +1824,7 @@
         <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>2572</v>
+        <v>4906</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1833,22 +1833,22 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>290.6635809214624</v>
+        <v>191.2082773776893</v>
       </c>
       <c r="K23" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="L23" t="n">
-        <v>570</v>
+        <v>530</v>
       </c>
       <c r="M23" t="n">
-        <v>126.1503559999255</v>
+        <v>10.08204199933971</v>
       </c>
       <c r="N23" t="n">
-        <v>1456.220934999692</v>
+        <v>1239.246555000136</v>
       </c>
       <c r="O23" t="n">
-        <v>21.59322051153143</v>
+        <v>41.14301244573974</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
@@ -1882,10 +1882,10 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G24" t="n">
-        <v>4923</v>
+        <v>8196</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1894,22 +1894,22 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>2714.134619197647</v>
+        <v>1156.890103463281</v>
       </c>
       <c r="K24" t="n">
-        <v>2600</v>
+        <v>1100</v>
       </c>
       <c r="L24" t="n">
-        <v>4000</v>
+        <v>2800</v>
       </c>
       <c r="M24" t="n">
-        <v>271.8974259996685</v>
+        <v>11.96608700047364</v>
       </c>
       <c r="N24" t="n">
-        <v>6288.057036999817</v>
+        <v>4650.954235001336</v>
       </c>
       <c r="O24" t="n">
-        <v>41.26637670453425</v>
+        <v>68.43340582900144</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
@@ -1943,10 +1943,10 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G25" t="n">
-        <v>4896</v>
+        <v>8616</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1955,22 +1955,22 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>9710.8166797635</v>
+        <v>2522.005538275666</v>
       </c>
       <c r="K25" t="n">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="L25" t="n">
-        <v>12000</v>
+        <v>5400</v>
       </c>
       <c r="M25" t="n">
-        <v>1208.814936999261</v>
+        <v>18.18550499956473</v>
       </c>
       <c r="N25" t="n">
-        <v>13091.27987899956</v>
+        <v>7924.065122000684</v>
       </c>
       <c r="O25" t="n">
-        <v>40.9262486676078</v>
+        <v>71.83191256219605</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
@@ -2007,7 +2007,7 @@
         <v>50</v>
       </c>
       <c r="G26" t="n">
-        <v>2538</v>
+        <v>4957</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -2016,22 +2016,22 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>324.9334645504563</v>
+        <v>192.8743321319337</v>
       </c>
       <c r="K26" t="n">
-        <v>260</v>
+        <v>160</v>
       </c>
       <c r="L26" t="n">
-        <v>550</v>
+        <v>510</v>
       </c>
       <c r="M26" t="n">
-        <v>122.138203000759</v>
+        <v>8.808614000372472</v>
       </c>
       <c r="N26" t="n">
-        <v>3511.551943999621</v>
+        <v>3820.819725000547</v>
       </c>
       <c r="O26" t="n">
-        <v>21.27410125718511</v>
+        <v>41.57040106313333</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2065,10 +2065,10 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G27" t="n">
-        <v>4686</v>
+        <v>8158</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -2077,22 +2077,22 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>2976.358505092825</v>
+        <v>1150.290196104075</v>
       </c>
       <c r="K27" t="n">
-        <v>2900</v>
+        <v>990</v>
       </c>
       <c r="L27" t="n">
-        <v>4600</v>
+        <v>2800</v>
       </c>
       <c r="M27" t="n">
-        <v>326.3911699996243</v>
+        <v>13.80985400101054</v>
       </c>
       <c r="N27" t="n">
-        <v>8880.769366000095</v>
+        <v>5843.95454299738</v>
       </c>
       <c r="O27" t="n">
-        <v>39.28464913441911</v>
+        <v>68.3000210556154</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2126,37 +2126,37 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G28" t="n">
-        <v>4987</v>
+        <v>8415</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>0.07130124777183601</v>
       </c>
       <c r="J28" t="n">
-        <v>9462.239501426113</v>
+        <v>2584.218952592274</v>
       </c>
       <c r="K28" t="n">
-        <v>9900</v>
+        <v>2200</v>
       </c>
       <c r="L28" t="n">
-        <v>11000</v>
+        <v>5400</v>
       </c>
       <c r="M28" t="n">
-        <v>1601.593557999877</v>
+        <v>3.051319999940461</v>
       </c>
       <c r="N28" t="n">
-        <v>15725.74061099931</v>
+        <v>8654.16466500028</v>
       </c>
       <c r="O28" t="n">
-        <v>41.63192049246334</v>
+        <v>70.61430010981178</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
+        <v>0.0503488770836447</v>
       </c>
       <c r="Q28" t="n">
         <v>2</v>
@@ -2190,7 +2190,7 @@
         <v>50</v>
       </c>
       <c r="G29" t="n">
-        <v>2356</v>
+        <v>2511</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -2199,22 +2199,22 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>509.5787934809038</v>
+        <v>345.7713445885885</v>
       </c>
       <c r="K29" t="n">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="L29" t="n">
-        <v>1100</v>
+        <v>680</v>
       </c>
       <c r="M29" t="n">
-        <v>178.9341020003121</v>
+        <v>134.837214000072</v>
       </c>
       <c r="N29" t="n">
-        <v>2566.110498999933</v>
+        <v>1345.842381000693</v>
       </c>
       <c r="O29" t="n">
-        <v>19.82207505498572</v>
+        <v>21.05188715117445</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2248,10 +2248,10 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G30" t="n">
-        <v>3954</v>
+        <v>4199</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -2260,22 +2260,22 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>3847.770278146439</v>
+        <v>2191.245934879485</v>
       </c>
       <c r="K30" t="n">
-        <v>3800</v>
+        <v>2100</v>
       </c>
       <c r="L30" t="n">
-        <v>5500</v>
+        <v>3300</v>
       </c>
       <c r="M30" t="n">
-        <v>531.9664170001488</v>
+        <v>367.1979870014184</v>
       </c>
       <c r="N30" t="n">
-        <v>9627.836168999693</v>
+        <v>5774.928037000791</v>
       </c>
       <c r="O30" t="n">
-        <v>33.13027750814875</v>
+        <v>35.13006755129004</v>
       </c>
       <c r="P30" t="n">
         <v>0</v>
@@ -2309,37 +2309,37 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G31" t="n">
-        <v>4432</v>
+        <v>3981</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>0.1758352172820899</v>
       </c>
       <c r="J31" t="n">
-        <v>10879.46813752915</v>
+        <v>5363.310673388613</v>
       </c>
       <c r="K31" t="n">
-        <v>11000</v>
+        <v>5000</v>
       </c>
       <c r="L31" t="n">
-        <v>13000</v>
+        <v>10000</v>
       </c>
       <c r="M31" t="n">
-        <v>1850.165803999971</v>
+        <v>2.735451000262401</v>
       </c>
       <c r="N31" t="n">
-        <v>15059.47390100027</v>
+        <v>15982.95562299972</v>
       </c>
       <c r="O31" t="n">
-        <v>37.09850605630296</v>
+        <v>33.42541604012995</v>
       </c>
       <c r="P31" t="n">
-        <v>0</v>
+        <v>0.058773652921605</v>
       </c>
       <c r="Q31" t="n">
         <v>2</v>
@@ -2373,7 +2373,7 @@
         <v>50</v>
       </c>
       <c r="G32" t="n">
-        <v>2550</v>
+        <v>2535</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -2382,22 +2382,22 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>316.6968367172556</v>
+        <v>327.3059481558278</v>
       </c>
       <c r="K32" t="n">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="L32" t="n">
-        <v>590</v>
+        <v>600</v>
       </c>
       <c r="M32" t="n">
-        <v>132.9148309996526</v>
+        <v>136.8486640003539</v>
       </c>
       <c r="N32" t="n">
-        <v>1015.008221000244</v>
+        <v>1056.163750999985</v>
       </c>
       <c r="O32" t="n">
-        <v>21.40883624096682</v>
+        <v>21.26633078129685</v>
       </c>
       <c r="P32" t="n">
         <v>0</v>
@@ -2431,10 +2431,10 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G33" t="n">
-        <v>4478</v>
+        <v>4220</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -2443,22 +2443,22 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>3151.670940313973</v>
+        <v>2160.602237813749</v>
       </c>
       <c r="K33" t="n">
-        <v>3100</v>
+        <v>2100</v>
       </c>
       <c r="L33" t="n">
-        <v>4700</v>
+        <v>3200</v>
       </c>
       <c r="M33" t="n">
-        <v>408.110700999714</v>
+        <v>517.7540590011631</v>
       </c>
       <c r="N33" t="n">
-        <v>7361.310508000315</v>
+        <v>5124.542711000686</v>
       </c>
       <c r="O33" t="n">
-        <v>37.53879193156863</v>
+        <v>35.33900449675799</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
@@ -2492,10 +2492,10 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G34" t="n">
-        <v>4577</v>
+        <v>4359</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -2504,22 +2504,22 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>10560.94507589335</v>
+        <v>4901.491026516851</v>
       </c>
       <c r="K34" t="n">
-        <v>11000</v>
+        <v>4800</v>
       </c>
       <c r="L34" t="n">
-        <v>12000</v>
+        <v>6700</v>
       </c>
       <c r="M34" t="n">
-        <v>1723.517123999954</v>
+        <v>1120.543047998581</v>
       </c>
       <c r="N34" t="n">
-        <v>13811.19311400016</v>
+        <v>9959.064340000625</v>
       </c>
       <c r="O34" t="n">
-        <v>38.10860790711043</v>
+        <v>36.44074658878257</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
@@ -2556,7 +2556,7 @@
         <v>50</v>
       </c>
       <c r="G35" t="n">
-        <v>2548</v>
+        <v>2508</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -2565,22 +2565,22 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>324.0206573359553</v>
+        <v>345.5456494066647</v>
       </c>
       <c r="K35" t="n">
-        <v>270</v>
+        <v>300</v>
       </c>
       <c r="L35" t="n">
-        <v>640</v>
+        <v>610</v>
       </c>
       <c r="M35" t="n">
-        <v>133.5762139997314</v>
+        <v>139.3599799994263</v>
       </c>
       <c r="N35" t="n">
-        <v>3765.626329000042</v>
+        <v>3659.002600999884</v>
       </c>
       <c r="O35" t="n">
-        <v>21.37458661125424</v>
+        <v>21.0266736440595</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
@@ -2614,10 +2614,10 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G36" t="n">
-        <v>4228</v>
+        <v>4149</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -2626,22 +2626,22 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>3465.258871412957</v>
+        <v>2233.616888937836</v>
       </c>
       <c r="K36" t="n">
-        <v>3200</v>
+        <v>2200</v>
       </c>
       <c r="L36" t="n">
-        <v>5900</v>
+        <v>3400</v>
       </c>
       <c r="M36" t="n">
-        <v>400.5781509995359</v>
+        <v>519.3338099998073</v>
       </c>
       <c r="N36" t="n">
-        <v>10657.89189100087</v>
+        <v>6327.618073000849</v>
       </c>
       <c r="O36" t="n">
-        <v>35.29140209127926</v>
+        <v>34.75165303209591</v>
       </c>
       <c r="P36" t="n">
         <v>0</v>
@@ -2675,10 +2675,10 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>520</v>
+        <v>260</v>
       </c>
       <c r="G37" t="n">
-        <v>4558</v>
+        <v>4378</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -2687,22 +2687,22 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>10624.65906421653</v>
+        <v>4863.241463538159</v>
       </c>
       <c r="K37" t="n">
-        <v>11000</v>
+        <v>4900</v>
       </c>
       <c r="L37" t="n">
-        <v>13000</v>
+        <v>6500</v>
       </c>
       <c r="M37" t="n">
-        <v>1620.69529099972</v>
+        <v>831.5197979991353</v>
       </c>
       <c r="N37" t="n">
-        <v>16445.43532999978</v>
+        <v>9135.438690000228</v>
       </c>
       <c r="O37" t="n">
-        <v>37.93007087286138</v>
+        <v>36.76884535582546</v>
       </c>
       <c r="P37" t="n">
         <v>0</v>

</xml_diff>